<commit_message>
默认输入改为CH2D3示例(C natural 1+H natural 2+D 3)
</commit_message>
<xml_diff>
--- a/ExactMass_Impurities.xlsx
+++ b/ExactMass_Impurities.xlsx
@@ -1848,7 +1848,11 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D3" s="8" t="n"/>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
       <c r="E3" s="8" t="n"/>
       <c r="F3" s="8" t="n"/>
       <c r="G3" s="8" t="n"/>
@@ -1886,10 +1890,14 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
+          <t>natural</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D4" s="8" t="n"/>
       <c r="E4" s="8" t="n"/>
       <c r="F4" s="8" t="n"/>
       <c r="G4" s="8" t="n"/>
@@ -1921,12 +1929,14 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="D5" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="9" t="n"/>
       <c r="E5" s="9" t="n"/>
       <c r="F5" s="9" t="n"/>
       <c r="G5" s="9" t="n"/>

</xml_diff>